<commit_message>
Fix Nutanix Customer Account step; prefill input template with tested models
Customer Account: browser code had a named helper that tsx wraps in __name(),
absent in the page; inlined, with a unit test that compiles src as tsx does.
OCA fills the account list only as a name is typed, so the step now types into
"Type to search..." and waits for the account instead of checking the list first.

The input template lists the 12 models run so far, with a Notes column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GGE6raah54XeD8ViTN2wo
</commit_message>
<xml_diff>
--- a/input/OCA-Input-Template.xlsx
+++ b/input/OCA-Input-Template.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L13"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -412,6 +412,7 @@
     <col min="9" max="9" width="22.83203125" customWidth="1"/>
     <col min="10" max="10" width="16.83203125" customWidth="1"/>
     <col min="11" max="11" width="9.83203125" customWidth="1"/>
+    <col min="12" max="12" width="90.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,13 +449,16 @@
       <c r="K1" t="str">
         <v>Enabled</v>
       </c>
+      <c r="L1" t="str">
+        <v>Notes</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>JOB-001</v>
       </c>
       <c r="B2" t="str">
-        <v>P75399-B21</v>
+        <v>P72176-B21</v>
       </c>
       <c r="C2" t="str">
         <v>Server</v>
@@ -482,6 +486,9 @@
       </c>
       <c r="K2" t="str">
         <v>Yes</v>
+      </c>
+      <c r="L2" t="str">
+        <v>DL360 Gen12. Passed end to end.</v>
       </c>
     </row>
     <row r="3">
@@ -489,10 +496,10 @@
         <v>JOB-002</v>
       </c>
       <c r="B3" t="str">
-        <v>P72176-B21</v>
+        <v>P72297-B21</v>
       </c>
       <c r="C3" t="str">
-        <v>Nutanix</v>
+        <v>Server</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -517,6 +524,9 @@
       </c>
       <c r="K3" t="str">
         <v>Yes</v>
+      </c>
+      <c r="L3" t="str">
+        <v>DL360-class. Passed end to end.</v>
       </c>
     </row>
     <row r="4">
@@ -524,10 +534,10 @@
         <v>JOB-003</v>
       </c>
       <c r="B4" t="str">
-        <v>S3V83A</v>
+        <v>P75219-B21</v>
       </c>
       <c r="C4" t="str">
-        <v>Solution</v>
+        <v>Server</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -552,6 +562,9 @@
       </c>
       <c r="K4" t="str">
         <v>Yes</v>
+      </c>
+      <c r="L4" t="str">
+        <v>DL320 Gen12. Passed end to end.</v>
       </c>
     </row>
     <row r="5">
@@ -559,10 +572,10 @@
         <v>JOB-004</v>
       </c>
       <c r="B5" t="str">
-        <v>S2U63A</v>
+        <v>P75220-B21</v>
       </c>
       <c r="C5" t="str">
-        <v>Storage</v>
+        <v>Server</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -588,17 +601,324 @@
       <c r="K5" t="str">
         <v>Yes</v>
       </c>
+      <c r="L5" t="str">
+        <v>DL320 Gen12. Passed end to end.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>JOB-005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>P75217-B21</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Server</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v>Random</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L6" t="str">
+        <v>DL320 Gen12. Failed on a boot device rule; repair added, retest.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>JOB-006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>P75218-B21</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Server</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>Random</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L7" t="str">
+        <v>DL320 Gen12. Failed on an OCP/processor rule; repair added, retest.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>JOB-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>P86628-B21</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Server</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v>Random</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L8" t="str">
+        <v>DL110 Gen12. Failed on the M.2 rule; fixed, retest.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>JOB-008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>P83540-B21</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Server</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v>Random</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L9" t="str">
+        <v>DL580 Gen12. Failed on Smart Chassis (old build); fixed, retest.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>JOB-009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>P75399-B21</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Server</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v>Random</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L10" t="str">
+        <v>DL580 Gen12 SFF. Failed on non-mandatory red icons; now only Processor/Memory block, retest.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>JOB-010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>P72176-B21</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Nutanix</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v>Random</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Nutanix DL360 G12. Failed in Customer Account; fixed, retest.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>JOB-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>S3V83A</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v>Random</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L12" t="str">
+        <v>dHCI solution. Wizard and Menu passed; server inside the solution added, retest.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>JOB-012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>S2U63A</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Server</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v>Random</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L13" t="str">
+        <v>DL380 Gen11 Data Solutions. Stopped at Billing Tier; capacity entry added, retest.</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G1"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -632,62 +952,16 @@
         <v>Sequence</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>JOB-001</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Processor</v>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v>random</v>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>JOB-001</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Memory</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v>random</v>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3">
-        <v>20</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -839,84 +1113,95 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Components sheet</v>
+        <v>Notes</v>
       </c>
       <c r="B14" t="str">
-        <v/>
+        <v>Optional</v>
       </c>
       <c r="C14" t="str">
-        <v>Optional. A model with no rows here gets random Processor, Memory, Smart Chassis and Power Supplies. Processor and Memory are always mandatory.</v>
+        <v>Free text for the team; not read by the tool.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Section</v>
+        <v>Components sheet</v>
       </c>
       <c r="B15" t="str">
-        <v>Required per row</v>
+        <v/>
       </c>
       <c r="C15" t="str">
-        <v>OCA Menu section title, e.g. Processor, Memory, Power Supplies.</v>
+        <v>Optional. A model with no rows here gets random Processor, Memory, Smart Chassis and Power Supplies. Processor and Memory are always mandatory.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Product Number</v>
+        <v>Section</v>
       </c>
       <c r="B16" t="str">
-        <v>Optional</v>
+        <v>Required per row</v>
       </c>
       <c r="C16" t="str">
-        <v>Product to select, e.g. P74509-B21. Blank with Random: any product.</v>
+        <v>OCA Menu section title, e.g. Processor, Memory, Power Supplies.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Quantity</v>
+        <v>Product Number</v>
       </c>
       <c r="B17" t="str">
         <v>Optional</v>
       </c>
       <c r="C17" t="str">
-        <v>Number to select.</v>
+        <v>Product to select, e.g. P74509-B21. Blank with Random: any product.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Selection Type</v>
+        <v>Quantity</v>
       </c>
       <c r="B18" t="str">
-        <v>radio / quantity / random / checkbox / configuration / automatic / default</v>
+        <v>Optional</v>
       </c>
       <c r="C18" t="str">
-        <v>How the product is selected; Random picks any allowed product.</v>
+        <v>Number to select.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Configuration Text</v>
+        <v>Selection Type</v>
       </c>
       <c r="B19" t="str">
-        <v>Optional</v>
+        <v>radio / quantity / random / checkbox / configuration / automatic / default</v>
       </c>
       <c r="C19" t="str">
-        <v>Configuration selection: the option text.</v>
+        <v>How the product is selected; Random picks any allowed product.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Sequence</v>
+        <v>Configuration Text</v>
       </c>
       <c r="B20" t="str">
         <v>Optional</v>
       </c>
       <c r="C20" t="str">
+        <v>Configuration selection: the option text.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Sequence</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Optional</v>
+      </c>
+      <c r="C21" t="str">
         <v>Order of the rows within a model (10, 20, 30...).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Country setting; open solutions searched by a word; wizard Server Qty and Menu picks follow OCA's ranges
- Country field (Excel, dashboard, template; blank = United States) set on the landing page by its label
- Search entries may match the Model Description; solutions prefer the Wizard card; templates never count
- dHCI Server Qty within the wizard's stated Min/Max; solution Menu picks follow the choice's quantity rule
- Input template row JOB-013: Arcus S3V83A in Saudi Arabia; change log and handoff updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GGE6raah54XeD8ViTN2wo
</commit_message>
<xml_diff>
--- a/input/OCA-Input-Template.xlsx
+++ b/input/OCA-Input-Template.xlsx
@@ -399,20 +399,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:M14"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="26.83203125" customWidth="1"/>
     <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="13.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="26.83203125" customWidth="1"/>
-    <col min="9" max="9" width="22.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="9.83203125" customWidth="1"/>
-    <col min="12" max="12" width="90.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="26.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="9.83203125" customWidth="1"/>
+    <col min="13" max="13" width="90.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -432,24 +433,27 @@
         <v>Customer Account</v>
       </c>
       <c r="F1" t="str">
+        <v>Country</v>
+      </c>
+      <c r="G1" t="str">
         <v>Service Type</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Server</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Integration Rack Part number</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Solution Name</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Generate End BOM</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Enabled</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -470,11 +474,11 @@
         <v/>
       </c>
       <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
         <v>Random</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
       <c r="H2" t="str">
         <v/>
       </c>
@@ -482,12 +486,15 @@
         <v/>
       </c>
       <c r="J2" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="K2" t="str">
         <v>Yes</v>
       </c>
       <c r="L2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M2" t="str">
         <v>DL360 Gen12. Passed end to end.</v>
       </c>
     </row>
@@ -508,11 +515,11 @@
         <v/>
       </c>
       <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
         <v>Random</v>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
       <c r="H3" t="str">
         <v/>
       </c>
@@ -520,12 +527,15 @@
         <v/>
       </c>
       <c r="J3" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="K3" t="str">
         <v>Yes</v>
       </c>
       <c r="L3" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M3" t="str">
         <v>DL360-class. Passed end to end.</v>
       </c>
     </row>
@@ -546,11 +556,11 @@
         <v/>
       </c>
       <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
         <v>Random</v>
       </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
       <c r="H4" t="str">
         <v/>
       </c>
@@ -558,12 +568,15 @@
         <v/>
       </c>
       <c r="J4" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="K4" t="str">
         <v>Yes</v>
       </c>
       <c r="L4" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M4" t="str">
         <v>DL320 Gen12. Passed end to end.</v>
       </c>
     </row>
@@ -584,11 +597,11 @@
         <v/>
       </c>
       <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
         <v>Random</v>
       </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
       <c r="H5" t="str">
         <v/>
       </c>
@@ -596,12 +609,15 @@
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="K5" t="str">
         <v>Yes</v>
       </c>
       <c r="L5" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M5" t="str">
         <v>DL320 Gen12. Passed end to end.</v>
       </c>
     </row>
@@ -622,11 +638,11 @@
         <v/>
       </c>
       <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
         <v>Random</v>
       </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
       <c r="H6" t="str">
         <v/>
       </c>
@@ -634,12 +650,15 @@
         <v/>
       </c>
       <c r="J6" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="K6" t="str">
         <v>Yes</v>
       </c>
       <c r="L6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M6" t="str">
         <v>DL320 Gen12. Failed on a boot device rule; repair added, retest.</v>
       </c>
     </row>
@@ -660,11 +679,11 @@
         <v/>
       </c>
       <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
         <v>Random</v>
       </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
       <c r="H7" t="str">
         <v/>
       </c>
@@ -672,12 +691,15 @@
         <v/>
       </c>
       <c r="J7" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="K7" t="str">
         <v>Yes</v>
       </c>
       <c r="L7" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M7" t="str">
         <v>DL320 Gen12. Failed on an OCP/processor rule; repair added, retest.</v>
       </c>
     </row>
@@ -698,11 +720,11 @@
         <v/>
       </c>
       <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
         <v>Random</v>
       </c>
-      <c r="G8" t="str">
-        <v/>
-      </c>
       <c r="H8" t="str">
         <v/>
       </c>
@@ -710,12 +732,15 @@
         <v/>
       </c>
       <c r="J8" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="K8" t="str">
         <v>Yes</v>
       </c>
       <c r="L8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M8" t="str">
         <v>DL110 Gen12. Failed on the M.2 rule; fixed, retest.</v>
       </c>
     </row>
@@ -736,11 +761,11 @@
         <v/>
       </c>
       <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
         <v>Random</v>
       </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
       <c r="H9" t="str">
         <v/>
       </c>
@@ -748,12 +773,15 @@
         <v/>
       </c>
       <c r="J9" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="K9" t="str">
         <v>Yes</v>
       </c>
       <c r="L9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M9" t="str">
         <v>DL580 Gen12. Failed on Smart Chassis (old build); fixed, retest.</v>
       </c>
     </row>
@@ -774,11 +802,11 @@
         <v/>
       </c>
       <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
         <v>Random</v>
       </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
       <c r="H10" t="str">
         <v/>
       </c>
@@ -786,12 +814,15 @@
         <v/>
       </c>
       <c r="J10" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="K10" t="str">
         <v>Yes</v>
       </c>
       <c r="L10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M10" t="str">
         <v>DL580 Gen12 SFF. Failed on non-mandatory red icons; now only Processor/Memory block, retest.</v>
       </c>
     </row>
@@ -812,11 +843,11 @@
         <v/>
       </c>
       <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
         <v>Random</v>
       </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
       <c r="H11" t="str">
         <v/>
       </c>
@@ -824,12 +855,15 @@
         <v/>
       </c>
       <c r="J11" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="K11" t="str">
         <v>Yes</v>
       </c>
       <c r="L11" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M11" t="str">
         <v>Nutanix DL360 G12. Failed in Customer Account; fixed, retest.</v>
       </c>
     </row>
@@ -850,11 +884,11 @@
         <v/>
       </c>
       <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
         <v>Random</v>
       </c>
-      <c r="G12" t="str">
-        <v/>
-      </c>
       <c r="H12" t="str">
         <v/>
       </c>
@@ -862,12 +896,15 @@
         <v/>
       </c>
       <c r="J12" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="K12" t="str">
         <v>Yes</v>
       </c>
       <c r="L12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M12" t="str">
         <v>dHCI solution. Wizard and Menu passed; server inside the solution added, retest.</v>
       </c>
     </row>
@@ -888,11 +925,11 @@
         <v/>
       </c>
       <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
         <v>Random</v>
       </c>
-      <c r="G13" t="str">
-        <v/>
-      </c>
       <c r="H13" t="str">
         <v/>
       </c>
@@ -900,18 +937,62 @@
         <v/>
       </c>
       <c r="J13" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="K13" t="str">
         <v>Yes</v>
       </c>
       <c r="L13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M13" t="str">
         <v>DL380 Gen11 Data Solutions. Stopped at Billing Tier; capacity entry added, retest.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>JOB-013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>S3V83A</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Solution</v>
+      </c>
+      <c r="D14" t="str">
+        <v>HPE GreenLake for PC3000 with Alletra Storage MP (Block)</v>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v>SAUDI ARABIA</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Random</v>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Arcus dHCI solution in Saudi Arabia (same product as JOB-011). New: Country; retest.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -961,7 +1042,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -1047,161 +1128,172 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Service Type</v>
+        <v>Country</v>
       </c>
       <c r="B8" t="str">
         <v>Optional</v>
       </c>
       <c r="C8" t="str">
-        <v>Random (default) or the service experience to select.</v>
+        <v>Landing page Country, as OCA lists it (e.g. SAUDI ARABIA) or its code (SA). Blank: UNITED STATES.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Server</v>
+        <v>Service Type</v>
       </c>
       <c r="B9" t="str">
         <v>Optional</v>
       </c>
       <c r="C9" t="str">
-        <v>Solution models: the server to pick in the Solution Wizard.</v>
+        <v>Random (default) or the service experience to select.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Integration Rack Part number</v>
+        <v>Server</v>
       </c>
       <c r="B10" t="str">
         <v>Optional</v>
       </c>
       <c r="C10" t="str">
-        <v>Blank: Standalone. Yes: any rack. Or the rack option text.</v>
+        <v>Solution models: the server to pick in the Solution Wizard.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Solution Name</v>
+        <v>Integration Rack Part number</v>
       </c>
       <c r="B11" t="str">
         <v>Optional</v>
       </c>
       <c r="C11" t="str">
-        <v>Solution models: the solution to pick in the Solution Wizard.</v>
+        <v>Blank: Standalone. Yes: any rack. Or the rack option text.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Generate End BOM</v>
+        <v>Solution Name</v>
       </c>
       <c r="B12" t="str">
-        <v>Yes / No</v>
+        <v>Optional</v>
       </c>
       <c r="C12" t="str">
-        <v>Default Yes.</v>
+        <v>Solution models: the solution to pick in the Solution Wizard.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Enabled</v>
+        <v>Generate End BOM</v>
       </c>
       <c r="B13" t="str">
         <v>Yes / No</v>
       </c>
       <c r="C13" t="str">
-        <v>Default Yes. No: the row is skipped.</v>
+        <v>Default Yes.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Notes</v>
+        <v>Enabled</v>
       </c>
       <c r="B14" t="str">
-        <v>Optional</v>
+        <v>Yes / No</v>
       </c>
       <c r="C14" t="str">
-        <v>Free text for the team; not read by the tool.</v>
+        <v>Default Yes. No: the row is skipped.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Components sheet</v>
+        <v>Notes</v>
       </c>
       <c r="B15" t="str">
-        <v/>
+        <v>Optional</v>
       </c>
       <c r="C15" t="str">
-        <v>Optional. A model with no rows here gets random Processor, Memory, Smart Chassis and Power Supplies. Processor and Memory are always mandatory.</v>
+        <v>Free text for the team; not read by the tool.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Section</v>
+        <v>Components sheet</v>
       </c>
       <c r="B16" t="str">
-        <v>Required per row</v>
+        <v/>
       </c>
       <c r="C16" t="str">
-        <v>OCA Menu section title, e.g. Processor, Memory, Power Supplies.</v>
+        <v>Optional. A model with no rows here gets random Processor, Memory, Smart Chassis and Power Supplies. Processor and Memory are always mandatory.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Product Number</v>
+        <v>Section</v>
       </c>
       <c r="B17" t="str">
-        <v>Optional</v>
+        <v>Required per row</v>
       </c>
       <c r="C17" t="str">
-        <v>Product to select, e.g. P74509-B21. Blank with Random: any product.</v>
+        <v>OCA Menu section title, e.g. Processor, Memory, Power Supplies.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Quantity</v>
+        <v>Product Number</v>
       </c>
       <c r="B18" t="str">
         <v>Optional</v>
       </c>
       <c r="C18" t="str">
-        <v>Number to select.</v>
+        <v>Product to select, e.g. P74509-B21. Blank with Random: any product.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Selection Type</v>
+        <v>Quantity</v>
       </c>
       <c r="B19" t="str">
-        <v>radio / quantity / random / checkbox / configuration / automatic / default</v>
+        <v>Optional</v>
       </c>
       <c r="C19" t="str">
-        <v>How the product is selected; Random picks any allowed product.</v>
+        <v>Number to select.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Configuration Text</v>
+        <v>Selection Type</v>
       </c>
       <c r="B20" t="str">
-        <v>Optional</v>
+        <v>radio / quantity / random / checkbox / configuration / automatic / default</v>
       </c>
       <c r="C20" t="str">
-        <v>Configuration selection: the option text.</v>
+        <v>How the product is selected; Random picks any allowed product.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Sequence</v>
+        <v>Configuration Text</v>
       </c>
       <c r="B21" t="str">
         <v>Optional</v>
       </c>
       <c r="C21" t="str">
+        <v>Configuration selection: the option text.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Sequence</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Optional</v>
+      </c>
+      <c r="C22" t="str">
         <v>Order of the rows within a model (10, 20, 30...).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Model Type "Arcus EMEA": a Solution preset with Saudi Arabia and the Arcus description
Preset Model Types are one table, MODEL_PRESETS, giving the route and the
Customer Account, search description and Country for blank Excel cells.
Nutanix moved into it unchanged. Dashboard list, template row JOB-014,
handoff and change log updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GGE6raah54XeD8ViTN2wo
</commit_message>
<xml_diff>
--- a/input/OCA-Input-Template.xlsx
+++ b/input/OCA-Input-Template.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -990,9 +990,50 @@
         <v>Arcus dHCI solution in Saudi Arabia (same product as JOB-011). New: Country; retest.</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>JOB-014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Private</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Arcus EMEA</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v>Random</v>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Arcus EMEA preset: Saudi Arabia and the Arcus description filled in. New; test.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1098,10 +1139,10 @@
         <v>Model Type</v>
       </c>
       <c r="B5" t="str">
-        <v>Server / Solution / Storage / Nutanix or blank</v>
+        <v>Server / Solution / Storage / Nutanix / Arcus EMEA or blank</v>
       </c>
       <c r="C5" t="str">
-        <v>Server: Menu tab. Solution: Solution Wizard. Storage: storage flow. Nutanix: Customer Account set to Nutanix in Advanced Settings, the search result containing "Nutanix" is opened, then the Server route. Blank: detected from OCA.</v>
+        <v>Server: Menu tab. Solution: Solution Wizard. Storage: storage flow. Nutanix: Customer Account set to Nutanix in Advanced Settings, the search result containing "Nutanix" is opened, then the Server route. Arcus EMEA: the Arcus solution (HPE GreenLake for PC3000 with Alletra Storage MP (Block)) in SAUDI ARABIA, built in its Wizard; Model Number is the search word, e.g. Private. Blank: detected from OCA.</v>
       </c>
     </row>
     <row r="6">
@@ -1112,7 +1153,7 @@
         <v>Optional</v>
       </c>
       <c r="C6" t="str">
-        <v>Text the OCA search result must contain, when the model has several results. Nutanix models use "Nutanix" when blank.</v>
+        <v>Text the OCA search result must contain, when the model has several results. Nutanix models use "Nutanix" when blank; Arcus EMEA uses the Arcus solution name.</v>
       </c>
     </row>
     <row r="7">
@@ -1134,7 +1175,7 @@
         <v>Optional</v>
       </c>
       <c r="C8" t="str">
-        <v>Landing page Country, as OCA lists it (e.g. SAUDI ARABIA) or its code (SA). Blank: UNITED STATES.</v>
+        <v>Landing page Country, as OCA lists it (e.g. SAUDI ARABIA) or its code (SA). Blank: UNITED STATES (Arcus EMEA: SAUDI ARABIA).</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Model Type "Simplivity Wizard": open the Wizard card, then Processor, Memory and what the wizard still asks for
A solution offered as both a CTO and a Wizard card opens the Wizard card. The
non-dHCI wizard picks Processor and Memory, then fills every dropdown still at
"Please make a selection." and raises quantities to the minimum its messages
state. HTML capture after the wizard. Template rows JOB-015, JOB-016.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GGE6raah54XeD8ViTN2wo
</commit_message>
<xml_diff>
--- a/input/OCA-Input-Template.xlsx
+++ b/input/OCA-Input-Template.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M17"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -1031,9 +1031,91 @@
         <v>Arcus EMEA preset: Saudi Arabia and the Arcus description filled in. New; test.</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>JOB-015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>S8J33A</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Simplivity Wizard</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v>Random</v>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M16" t="str">
+        <v>SimpliVity 380 Gen12 in its Wizard. New; test.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>JOB-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>S2V31A</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Simplivity Wizard</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v>Random</v>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M17" t="str">
+        <v>SimpliVity 325 Gen11 in its Wizard. New; test.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1139,10 +1221,10 @@
         <v>Model Type</v>
       </c>
       <c r="B5" t="str">
-        <v>Server / Solution / Storage / Nutanix / Arcus EMEA or blank</v>
+        <v>Server / Solution / Storage / Nutanix / Arcus EMEA / Simplivity Wizard or blank</v>
       </c>
       <c r="C5" t="str">
-        <v>Server: Menu tab. Solution: Solution Wizard. Storage: storage flow. Nutanix: Customer Account set to Nutanix in Advanced Settings, the search result containing "Nutanix" is opened, then the Server route. Arcus EMEA: the Arcus solution (HPE GreenLake for PC3000 with Alletra Storage MP (Block)) in SAUDI ARABIA, built in its Wizard; Model Number is the search word, e.g. Private. Blank: detected from OCA.</v>
+        <v>Server: Menu tab. Solution: Solution Wizard. Storage: storage flow. Nutanix: Customer Account set to Nutanix in Advanced Settings, the search result containing "Nutanix" is opened, then the Server route. Arcus EMEA: the Arcus solution (HPE GreenLake for PC3000 with Alletra Storage MP (Block)) in SAUDI ARABIA, built in its Wizard; Model Number is the search word, e.g. Private. Simplivity Wizard: the Wizard card of the model is opened (not its CTO card); Processor and Memory are picked, then every wizard dropdown still asking for a selection, at the minimum quantity its messages state. Blank: detected from OCA.</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Model Types "Alletra 4000" and "Alletra 5000": wizards searched by a word, completed tab by tab
The Solution Wizard now configures a wizard shown without a Solution Wizard tab
(.wizard_content), works through the wizard's own tabs, fills mandatory dropdowns
before Processor first (the base Alletra Storage Server) and keeps the Processor
and Memory that base model set. A wizard with no Processor or Memory dropdown (a
storage array) passes. Template rows JOB-017, JOB-018.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PpSUhjoTe22Zt5ZGAeFV5f
</commit_message>
<xml_diff>
--- a/input/OCA-Input-Template.xlsx
+++ b/input/OCA-Input-Template.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M19"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -1113,9 +1113,91 @@
         <v>SimpliVity 325 Gen11 in its Wizard. New; test.</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>JOB-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>4000</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Alletra 4000</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v>Random</v>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M18" t="str">
+        <v>HPE Alletra Storage Servers in their wizard. New; test.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>JOB-018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>alletra</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Alletra 5000</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v>Random</v>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M19" t="str">
+        <v>HPE Alletra 5000 array in the Alletra5000Sol Wizard. New; test.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1221,10 +1303,10 @@
         <v>Model Type</v>
       </c>
       <c r="B5" t="str">
-        <v>Server / Solution / Storage / Nutanix / Arcus EMEA / Simplivity Wizard or blank</v>
+        <v>Server / Solution / Storage / Nutanix / Arcus EMEA / Simplivity Wizard / Alletra 4000 / Alletra 5000 or blank</v>
       </c>
       <c r="C5" t="str">
-        <v>Server: Menu tab. Solution: Solution Wizard. Storage: storage flow. Nutanix: Customer Account set to Nutanix in Advanced Settings, the search result containing "Nutanix" is opened, then the Server route. Arcus EMEA: the Arcus solution (HPE GreenLake for PC3000 with Alletra Storage MP (Block)) in SAUDI ARABIA, built in its Wizard; Model Number is the search word, e.g. Private. Simplivity Wizard: the Wizard card of the model is opened (not its CTO card); Processor and Memory are picked, then every wizard dropdown still asking for a selection, at the minimum quantity its messages state. Blank: detected from OCA.</v>
+        <v>Server: Menu tab. Solution: Solution Wizard. Storage: storage flow. Nutanix: Customer Account set to Nutanix in Advanced Settings, the search result containing "Nutanix" is opened, then the Server route. Arcus EMEA: the Arcus solution (HPE GreenLake for PC3000 with Alletra Storage MP (Block)) in SAUDI ARABIA, built in its Wizard; Model Number is the search word, e.g. Private. Simplivity Wizard: the Wizard card of the model is opened (not its CTO card); Processor and Memory are picked, then every wizard dropdown still asking for a selection, at the minimum quantity its messages state. Alletra 4000 / Alletra 5000: the "HPE Alletra Storage Servers" / "HPE Alletra 5000" search result (Model Number is the search word, e.g. 4000 / alletra), built in its wizard: the base model first, then each wizard tab's mandatory dropdowns. Blank: detected from OCA.</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Alletra 4000/5000 verified on OCA: change log and template notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PpSUhjoTe22Zt5ZGAeFV5f
</commit_message>
<xml_diff>
--- a/input/OCA-Input-Template.xlsx
+++ b/input/OCA-Input-Template.xlsx
@@ -1151,7 +1151,7 @@
         <v>Yes</v>
       </c>
       <c r="M18" t="str">
-        <v>HPE Alletra Storage Servers in their wizard. New; test.</v>
+        <v>HPE Alletra Storage Servers in their wizard. Passed (2026-10-22).</v>
       </c>
     </row>
     <row r="19">
@@ -1192,7 +1192,7 @@
         <v>Yes</v>
       </c>
       <c r="M19" t="str">
-        <v>HPE Alletra 5000 array in the Alletra5000Sol Wizard. New; test.</v>
+        <v>HPE Alletra 5000 array in the Alletra5000Sol Wizard. Passed (2026-10-22).</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Storage S1F24A (GreenLake for File): Site Survey, optional node sections; lowest-power CPU when all exceed 270W
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PpSUhjoTe22Zt5ZGAeFV5f
</commit_message>
<xml_diff>
--- a/input/OCA-Input-Template.xlsx
+++ b/input/OCA-Input-Template.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M21"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -1195,9 +1195,91 @@
         <v>HPE Alletra 5000 array in the Alletra5000Sol Wizard. Passed (2026-10-22).</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>JOB-019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>S1F24A</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Storage</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v>Random</v>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M20" t="str">
+        <v>HPE GreenLake for File ("razercrestsol" CTO): Cloud Connectivity, Site Survey, Capacity. New; test.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>JOB-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>P97048-B21</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Server</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v>Random</v>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M21" t="str">
+        <v>DL585a Gen13: every processor over 270W; the lowest power is taken. Retest.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1306,7 +1388,7 @@
         <v>Server / Solution / Storage / Nutanix / Arcus EMEA / Simplivity Wizard / Alletra 4000 / Alletra 5000 or blank</v>
       </c>
       <c r="C5" t="str">
-        <v>Server: Menu tab. Solution: Solution Wizard. Storage: storage flow. Nutanix: Customer Account set to Nutanix in Advanced Settings, the search result containing "Nutanix" is opened, then the Server route. Arcus EMEA: the Arcus solution (HPE GreenLake for PC3000 with Alletra Storage MP (Block)) in SAUDI ARABIA, built in its Wizard; Model Number is the search word, e.g. Private. Simplivity Wizard: the Wizard card of the model is opened (not its CTO card); Processor and Memory are picked, then every wizard dropdown still asking for a selection, at the minimum quantity its messages state. Alletra 4000 / Alletra 5000: the "HPE Alletra Storage Servers" / "HPE Alletra 5000" search result (Model Number is the search word, e.g. 4000 / alletra), built in its wizard: the base model first, then each wizard tab's mandatory dropdowns. Blank: detected from OCA.</v>
+        <v>Server: Menu tab. Solution: Solution Wizard. Storage: storage flow (Cloud Connectivity, Controller Nodes or Site Survey, Capacity; e.g. S1F24A). Nutanix: Customer Account set to Nutanix in Advanced Settings, the search result containing "Nutanix" is opened, then the Server route. Arcus EMEA: the Arcus solution (HPE GreenLake for PC3000 with Alletra Storage MP (Block)) in SAUDI ARABIA, built in its Wizard; Model Number is the search word, e.g. Private. Simplivity Wizard: the Wizard card of the model is opened (not its CTO card); Processor and Memory are picked, then every wizard dropdown still asking for a selection, at the minimum quantity its messages state. Alletra 4000 / Alletra 5000: the "HPE Alletra Storage Servers" / "HPE Alletra 5000" search result (Model Number is the search word, e.g. 4000 / alletra), built in its wizard: the base model first, then each wizard tab's mandatory dropdowns. Blank: detected from OCA.</v>
       </c>
     </row>
     <row r="6">

</xml_diff>